<commit_message>
v0.6.5: jiufang Brand from B-column amazon title, first word before space
</commit_message>
<xml_diff>
--- a/templates/九方-模版.xlsx
+++ b/templates/九方-模版.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="31900" windowHeight="17260"/>
+    <workbookView windowHeight="11600"/>
   </bookViews>
   <sheets>
     <sheet name="下单模板" sheetId="1" r:id="rId1"/>
@@ -3326,7 +3326,7 @@
       <c r="G3" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="55" t="s">
+      <c r="H3" s="53" t="s">
         <v>17</v>
       </c>
       <c r="I3" s="55" t="s">

</xml_diff>

<commit_message>
v0.6.5: fix country code GB (not UK) mapping to GBP
</commit_message>
<xml_diff>
--- a/templates/九方-模版.xlsx
+++ b/templates/九方-模版.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="11600"/>
+    <workbookView windowHeight="10800"/>
   </bookViews>
   <sheets>
     <sheet name="下单模板" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="142">
   <si>
     <t>COMMERCIAL INVOICE &amp; Packing List</t>
   </si>
@@ -549,9 +549,6 @@
   </si>
   <si>
     <t>蜡烛</t>
-  </si>
-  <si>
-    <t>MSCandle</t>
   </si>
   <si>
     <t>92%植物混合蜡+8%的香精</t>
@@ -1667,13 +1664,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="微软雅黑"/>
+      <name val="宋体"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="宋体"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
@@ -2255,7 +2252,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2426,6 +2423,9 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="6" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -2437,6 +2437,9 @@
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="23" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3390,31 +3393,29 @@
       <c r="G4" s="57" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="57" t="s">
+      <c r="H4" s="57"/>
+      <c r="I4" s="58" t="s">
         <v>36</v>
       </c>
-      <c r="I4" s="57" t="s">
+      <c r="J4" s="57" t="s">
         <v>37</v>
-      </c>
-      <c r="J4" s="57" t="s">
-        <v>38</v>
       </c>
       <c r="K4" s="57">
         <v>3406000090</v>
       </c>
-      <c r="L4" s="58"/>
+      <c r="L4" s="59"/>
       <c r="M4" s="57" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" s="57" t="s">
         <v>39</v>
-      </c>
-      <c r="N4" s="57" t="s">
-        <v>40</v>
       </c>
       <c r="O4" s="56"/>
       <c r="P4" s="57" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q4" s="57" t="s">
         <v>41</v>
-      </c>
-      <c r="Q4" s="57" t="s">
-        <v>42</v>
       </c>
       <c r="R4" s="57"/>
       <c r="S4" s="56"/>
@@ -3427,44 +3428,42 @@
     <row r="5" ht="50" customHeight="1" spans="1:24">
       <c r="A5" s="56"/>
       <c r="B5" s="56"/>
-      <c r="C5" s="59"/>
+      <c r="C5" s="60"/>
       <c r="D5" s="56"/>
       <c r="E5" s="56"/>
-      <c r="F5" s="60" t="s">
+      <c r="F5" s="61" t="s">
+        <v>42</v>
+      </c>
+      <c r="G5" s="61" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="60" t="s">
+      <c r="H5" s="62"/>
+      <c r="I5" s="63" t="s">
         <v>44</v>
       </c>
-      <c r="H5" s="61" t="s">
-        <v>36</v>
-      </c>
-      <c r="I5" s="61" t="s">
+      <c r="J5" s="62" t="s">
+        <v>37</v>
+      </c>
+      <c r="K5" s="61">
+        <v>3307490000</v>
+      </c>
+      <c r="L5" s="64"/>
+      <c r="M5" s="64" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" s="64" t="s">
+        <v>39</v>
+      </c>
+      <c r="O5" s="56"/>
+      <c r="P5" s="64" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q5" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="J5" s="61" t="s">
-        <v>38</v>
-      </c>
-      <c r="K5" s="60">
-        <v>3307490000</v>
-      </c>
-      <c r="L5" s="62"/>
-      <c r="M5" s="62" t="s">
-        <v>39</v>
-      </c>
-      <c r="N5" s="62" t="s">
-        <v>40</v>
-      </c>
-      <c r="O5" s="56"/>
-      <c r="P5" s="62" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q5" s="62" t="s">
-        <v>46</v>
-      </c>
-      <c r="R5" s="63"/>
-      <c r="S5" s="62"/>
-      <c r="T5" s="63"/>
+      <c r="R5" s="65"/>
+      <c r="S5" s="64"/>
+      <c r="T5" s="65"/>
       <c r="U5" s="56"/>
       <c r="V5" s="56"/>
       <c r="W5" s="56"/>
@@ -3505,7 +3504,7 @@
   <sheetData>
     <row r="1" ht="28.8" spans="1:24">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3579,7 +3578,7 @@
       <c r="Q3" s="2"/>
       <c r="R3" s="2"/>
       <c r="S3" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="T3" s="7" t="s">
         <v>9</v>
@@ -3591,286 +3590,286 @@
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:24">
       <c r="A4" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="G4" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="H4" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="I4" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="J4" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="J4" s="11" t="s">
+      <c r="K4" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="L4" s="11" t="s">
         <v>59</v>
-      </c>
-      <c r="L4" s="11" t="s">
-        <v>60</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>22</v>
       </c>
       <c r="N4" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="O4" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="P4" s="11" t="s">
         <v>62</v>
-      </c>
-      <c r="P4" s="11" t="s">
-        <v>63</v>
       </c>
       <c r="Q4" s="11" t="s">
         <v>26</v>
       </c>
       <c r="R4" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="S4" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="S4" s="9" t="s">
+      <c r="T4" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="T4" s="11" t="s">
+      <c r="U4" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="U4" s="9" t="s">
+      <c r="V4" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="V4" s="9" t="s">
+      <c r="W4" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="W4" s="9" t="s">
+      <c r="X4" s="9" t="s">
         <v>69</v>
-      </c>
-      <c r="X4" s="9" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:24">
       <c r="A5" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="C5" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="D5" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="E5" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="F5" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="G5" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="H5" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="I5" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="I5" s="15" t="s">
+      <c r="J5" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="K5" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="K5" s="12" t="s">
+      <c r="L5" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="L5" s="17" t="s">
+      <c r="M5" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="N5" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="M5" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="N5" s="15" t="s">
+      <c r="O5" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="O5" s="12" t="s">
-        <v>84</v>
-      </c>
       <c r="P5" s="15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q5" s="12"/>
       <c r="R5" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="S5" s="12" t="s">
         <v>85</v>
-      </c>
-      <c r="S5" s="12" t="s">
-        <v>86</v>
       </c>
       <c r="T5" s="19"/>
       <c r="U5" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="V5" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="V5" s="12" t="s">
+      <c r="W5" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="W5" s="12" t="s">
+      <c r="X5" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="X5" s="13" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:24">
       <c r="A6" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="13" t="s">
+      <c r="D6" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="E6" s="12" t="s">
+      <c r="F6" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="J6" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="L6" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="M6" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="N6" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="O6" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="F6" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="H6" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="I6" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="J6" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="K6" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="L6" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="M6" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="N6" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="O6" s="12" t="s">
-        <v>94</v>
-      </c>
       <c r="P6" s="15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q6" s="12"/>
       <c r="R6" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="S6" s="12" t="s">
         <v>85</v>
-      </c>
-      <c r="S6" s="12" t="s">
-        <v>86</v>
       </c>
       <c r="T6" s="19"/>
       <c r="U6" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="V6" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="V6" s="12" t="s">
+      <c r="W6" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="W6" s="12" t="s">
+      <c r="X6" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="X6" s="13" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:24">
       <c r="A7" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="C7" s="20" t="s">
+      <c r="D7" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="E7" s="12" t="s">
+      <c r="F7" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="F7" s="21" t="s">
+      <c r="G7" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="G7" s="22" t="s">
+      <c r="H7" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="H7" s="15" t="s">
+      <c r="I7" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="J7" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="I7" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="J7" s="16" t="s">
+      <c r="K7" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="L7" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="K7" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="L7" s="17" t="s">
+      <c r="M7" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="N7" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="M7" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="N7" s="15" t="s">
+      <c r="O7" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="O7" s="12" t="s">
-        <v>104</v>
-      </c>
       <c r="P7" s="15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q7" s="12"/>
       <c r="R7" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="S7" s="12" t="s">
         <v>105</v>
-      </c>
-      <c r="S7" s="12" t="s">
-        <v>106</v>
       </c>
       <c r="T7" s="23"/>
       <c r="U7" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="V7" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="V7" s="12" t="s">
+      <c r="W7" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="X7" s="13" t="s">
         <v>108</v>
-      </c>
-      <c r="W7" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="X7" s="13" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:24">
@@ -3879,47 +3878,47 @@
       <c r="C8" s="24"/>
       <c r="D8" s="14"/>
       <c r="E8" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="F8" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="F8" s="25" t="s">
+      <c r="G8" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="G8" s="22" t="s">
+      <c r="H8" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="I8" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="I8" s="21" t="s">
+      <c r="J8" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="J8" s="13" t="s">
+      <c r="K8" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="L8" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="L8" s="17" t="s">
+      <c r="M8" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="N8" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="M8" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="N8" s="13" t="s">
+      <c r="O8" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="O8" s="13" t="s">
-        <v>119</v>
-      </c>
       <c r="P8" s="26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="Q8" s="27"/>
       <c r="R8" s="28">
         <v>36.24</v>
       </c>
       <c r="S8" s="13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="T8" s="29"/>
       <c r="U8" s="12"/>
@@ -3929,10 +3928,10 @@
     </row>
     <row r="9" ht="17.6" spans="1:24">
       <c r="A9" s="30" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C9" s="31"/>
       <c r="D9" s="31"/>
@@ -3959,10 +3958,10 @@
     </row>
     <row r="10" ht="17.6" spans="1:24">
       <c r="A10" s="35" t="s">
+        <v>121</v>
+      </c>
+      <c r="B10" s="36" t="s">
         <v>122</v>
-      </c>
-      <c r="B10" s="36" t="s">
-        <v>123</v>
       </c>
       <c r="C10" s="37"/>
       <c r="D10" s="37"/>
@@ -3989,10 +3988,10 @@
     </row>
     <row r="11" ht="17.6" spans="1:24">
       <c r="A11" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="B11" s="36" t="s">
         <v>124</v>
-      </c>
-      <c r="B11" s="36" t="s">
-        <v>125</v>
       </c>
       <c r="C11" s="37"/>
       <c r="D11" s="37"/>
@@ -4019,10 +4018,10 @@
     </row>
     <row r="12" ht="17.6" spans="1:24">
       <c r="A12" s="35" t="s">
+        <v>125</v>
+      </c>
+      <c r="B12" s="36" t="s">
         <v>126</v>
-      </c>
-      <c r="B12" s="36" t="s">
-        <v>127</v>
       </c>
       <c r="C12" s="37"/>
       <c r="D12" s="37"/>
@@ -4049,10 +4048,10 @@
     </row>
     <row r="13" ht="18" spans="1:24">
       <c r="A13" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="B13" s="36" t="s">
         <v>128</v>
-      </c>
-      <c r="B13" s="36" t="s">
-        <v>129</v>
       </c>
       <c r="C13" s="37"/>
       <c r="D13" s="37"/>
@@ -4079,10 +4078,10 @@
     </row>
     <row r="14" ht="17.6" spans="1:24">
       <c r="A14" s="35" t="s">
+        <v>129</v>
+      </c>
+      <c r="B14" s="36" t="s">
         <v>130</v>
-      </c>
-      <c r="B14" s="36" t="s">
-        <v>131</v>
       </c>
       <c r="C14" s="37"/>
       <c r="D14" s="37"/>
@@ -4109,10 +4108,10 @@
     </row>
     <row r="15" ht="17.6" spans="1:24">
       <c r="A15" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B15" s="36" t="s">
         <v>132</v>
-      </c>
-      <c r="B15" s="36" t="s">
-        <v>133</v>
       </c>
       <c r="C15" s="37"/>
       <c r="D15" s="37"/>
@@ -4139,10 +4138,10 @@
     </row>
     <row r="16" ht="17.6" spans="1:24">
       <c r="A16" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" s="36" t="s">
         <v>134</v>
-      </c>
-      <c r="B16" s="36" t="s">
-        <v>135</v>
       </c>
       <c r="C16" s="36"/>
       <c r="D16" s="36"/>
@@ -4169,10 +4168,10 @@
     </row>
     <row r="17" ht="18" spans="1:24">
       <c r="A17" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="B17" s="36" t="s">
         <v>136</v>
-      </c>
-      <c r="B17" s="36" t="s">
-        <v>137</v>
       </c>
       <c r="C17" s="37"/>
       <c r="D17" s="37"/>
@@ -4199,10 +4198,10 @@
     </row>
     <row r="18" ht="17.6" spans="1:24">
       <c r="A18" s="35" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B18" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C18" s="37"/>
       <c r="D18" s="37"/>
@@ -4229,10 +4228,10 @@
     </row>
     <row r="19" ht="17.6" spans="1:24">
       <c r="A19" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="B19" s="38" t="s">
         <v>139</v>
-      </c>
-      <c r="B19" s="38" t="s">
-        <v>140</v>
       </c>
       <c r="C19" s="39"/>
       <c r="D19" s="39"/>
@@ -4259,10 +4258,10 @@
     </row>
     <row r="20" ht="17.6" spans="1:24">
       <c r="A20" s="35" t="s">
+        <v>140</v>
+      </c>
+      <c r="B20" s="40" t="s">
         <v>141</v>
-      </c>
-      <c r="B20" s="40" t="s">
-        <v>142</v>
       </c>
       <c r="C20" s="41"/>
       <c r="D20" s="41"/>

</xml_diff>